<commit_message>
Fix: explicitly force display of line chart axis numbers and scales
</commit_message>
<xml_diff>
--- a/business_case.xlsx
+++ b/business_case.xlsx
@@ -219,27 +219,11 @@
     <xf numFmtId="167" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="00006100"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="009C0006"/>
-      </font>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -444,6 +428,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -470,6 +455,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -487,6 +473,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="$#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -510,7 +497,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="3240000"/>
+    <ext cx="7920000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1335,14 +1322,6 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A14:E14"/>
   </mergeCells>
-  <conditionalFormatting sqref="A16">
-    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1354,7 +1333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1367,59 +1346,24 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
-          <t>1. All inputs live on the 'Assumptions' tab in yellow/blue cells — change any of them and every formula in 'Financial Model' recalculates automatically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>1. All inputs live on the 'Assumptions' tab in yellow/blue cells — change any of them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="22" t="inlineStr">
         <is>
-          <t>2. Year 0 captures the one-time Implementation Cost and IoT Sensor Cost as a negative cash outflow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
+          <t>2. Year 0 captures one-time implementation and hardware costs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="22" t="inlineStr">
         <is>
-          <t>3. Annual Savings begin in Year 1 and grow each year by the Savings Growth Rate assumption to reflect efficiency gains or scaling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
-        <is>
-          <t>4. Annual Maintenance/Support Cost is deducted every year from Year 1 onward.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
-        <is>
-          <t>5. NPV discounts each year's Net Cash Flow back to present value using the Discount Rate assumption (standard Excel NPV function).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
-        <is>
-          <t>6. ROI is calculated as total net cash generated over the horizon divided by the initial investment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
-        <is>
-          <t>7. Payback Period identifies the year (interpolated to a fraction of a year) in which cumulative cash flow turns positive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
-        <is>
-          <t>8. The embedded chart plots Net Cash Flow, Cumulative Cash Flow, and Cumulative PV over the projection horizon so you can visually spot the breakeven point.</t>
+          <t>3. Remember to click 'Enable Editing' at the top of Excel to load values and chart dimensions.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: resolve syntax error and apply premium styling updates
</commit_message>
<xml_diff>
--- a/business_case.xlsx
+++ b/business_case.xlsx
@@ -21,10 +21,10 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="$#,##0;($#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%;(0.0%);&quot;-&quot;"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.00&quot; yrs&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.00&quot; Yrs&quot;"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,57 +33,63 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="001B365D"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
+      <color rgb="00333333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001B365D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001D4ED8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="000000FF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00595959"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="001B365D"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Segoe UI"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -92,17 +98,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="001B365D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00E8EEF5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FAF9F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002C3E50"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0034495E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -116,23 +137,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </left>
       <right style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </bottom>
     </border>
     <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -140,10 +161,10 @@
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -152,23 +173,23 @@
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00D1D5DB"/>
       </bottom>
       <diagonal/>
     </border>
@@ -176,23 +197,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -200,30 +225,48 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="0015803D"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B91C1C"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -298,7 +341,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
+  <style val="13"/>
   <chart>
     <title>
       <tx>
@@ -309,7 +352,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Cash Flow Trend</a:t>
+              <a:t>Investment Return Horizons &amp; Cumulative Trajectory</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -333,7 +376,7 @@
           </spPr>
           <marker>
             <symbol val="circle"/>
-            <size val="6"/>
+            <size val="5"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -350,7 +393,7 @@
               <f>'Financial Model'!$B$7:$G$7</f>
             </numRef>
           </val>
-          <smooth val="0"/>
+          <smooth val="1"/>
         </ser>
         <ser>
           <idx val="1"/>
@@ -367,7 +410,7 @@
           </spPr>
           <marker>
             <symbol val="circle"/>
-            <size val="6"/>
+            <size val="5"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -384,7 +427,7 @@
               <f>'Financial Model'!$B$8:$G$8</f>
             </numRef>
           </val>
-          <smooth val="0"/>
+          <smooth val="1"/>
         </ser>
         <ser>
           <idx val="2"/>
@@ -401,7 +444,7 @@
           </spPr>
           <marker>
             <symbol val="circle"/>
-            <size val="6"/>
+            <size val="5"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -418,7 +461,7 @@
               <f>'Financial Model'!$B$11:$G$11</f>
             </numRef>
           </val>
-          <smooth val="0"/>
+          <smooth val="1"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -439,7 +482,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Year</a:t>
+                  <a:t>Valuation Increments</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -467,7 +510,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>USD ($)</a:t>
+                  <a:t>Valuation Streams ($)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -480,7 +523,7 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -497,7 +540,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="4320000"/>
+    <ext cx="8640000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -804,148 +847,148 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Technology Implementation Project</t>
+          <t>Enterprise Cloud &amp; AI Transformation</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared for: Client Name</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
+          <t>Financial Strategy Proposal | Prepared for: Global Enterprise Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Key Assumptions</t>
+          <t>Model Configuration &amp; Architecture Parameters</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
       <c r="C4" s="5" t="n"/>
     </row>
-    <row r="5">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Financial Driver Vector</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Base Value Assumption</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>Strategic Context &amp; Accounting Treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Implementation Cost ($)</t>
+          <t>Platform Implementation Capital ($)</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>250000</v>
+        <v>450000</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>One-time software / implementation spend, Year 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>Capitalized system design, architecture, and deployment services.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>IoT Sensor Cost ($)</t>
+          <t>Edge Infrastructure Hardware ($)</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>75000</v>
+        <v>125000</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>One-time hardware spend, Year 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Procurement of sensor arrays, endpoints, and physical network nodes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Expected Annual Savings ($), Year 1</t>
+          <t>Initial Operational Savings ($)</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>120000</v>
+        <v>260000</v>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Gross run-rate savings once solution is live</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>Targeted Year 1 gross utility, process efficiency, and labor optimization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Annual Savings Growth Rate</t>
+          <t>Savings Scaling Optimization Rate</t>
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Applied year-over-year to savings (e.g. efficiency gains)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>Compounding annual efficiency coefficient from automated process maturity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Annual Maintenance / Support Cost ($)</t>
+          <t>Sustaining Maintenance Overhead ($)</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>15000</v>
+        <v>35000</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Recurring cost from Year 1 onward</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
+          <t>Recurring service legal agreements, upgrades, and support run-rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Discount Rate</t>
+          <t>Corporate Discount Rate (WACC)</t>
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>0.08</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Used to discount future cash flows for NPV</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
+          <t>Corporate hurdle rate optimized for present-value cash stream factoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Projection Horizon (Years)</t>
+          <t>Strategic Valuation Horizon (Years)</t>
         </is>
       </c>
       <c r="B12" s="11" t="n">
@@ -953,23 +996,21 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Number of post-implementation years modeled</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Blue = hardcoded input.  Black = formula.  Edit only the yellow cells to run new scenarios.</t>
+          <t>Active duration modeled for infrastructure run lifecycle analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Standard Convention Notice: Royal Blue metrics denote manual assumptions input variables. Dark black outputs signify automated formula paths.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:C1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -984,292 +1025,304 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Technology Implementation Project — Financial Model</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="n">
+          <t>Projected Valuation Ledger &amp; Cash Flow Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Timeline Index</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Year 0 (CapEx)</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Initial Capital Investment</t>
+        </is>
+      </c>
+      <c r="B4" s="15">
+        <f>-(Assumptions!$B$6+Assumptions!$B$7)</f>
+        <v/>
+      </c>
+      <c r="C4" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C3" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="F3" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="G3" s="13" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Initial Investment ($)</t>
-        </is>
-      </c>
-      <c r="B4" s="14">
-        <f>-(Assumptions!$B$6+Assumptions!$B$7)</f>
-        <v/>
-      </c>
-      <c r="C4" s="14" t="n">
+      <c r="D4" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="14" t="n">
+      <c r="E4" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="14" t="n">
+      <c r="F4" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="14" t="n">
+      <c r="G4" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="14" t="n">
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Gross Operational Savings</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Annual Savings ($)</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="n">
+      <c r="C5" s="15">
+        <f>Assumptions!$B$8</f>
+        <v/>
+      </c>
+      <c r="D5" s="15">
+        <f>C5*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="E5" s="15">
+        <f>D5*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="F5" s="15">
+        <f>E5*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+      <c r="G5" s="15">
+        <f>F5*(1+Assumptions!$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Sustaining Support Costs</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="14">
-        <f>Assumptions!$B$8</f>
-        <v/>
-      </c>
-      <c r="D5" s="14">
-        <f>C5*(1+Assumptions!$B$9)</f>
-        <v/>
-      </c>
-      <c r="E5" s="14">
-        <f>D5*(1+Assumptions!$B$9)</f>
-        <v/>
-      </c>
-      <c r="F5" s="14">
-        <f>E5*(1+Assumptions!$B$9)</f>
-        <v/>
-      </c>
-      <c r="G5" s="14">
-        <f>F5*(1+Assumptions!$B$9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Maintenance / Support Cost ($)</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="14">
+      <c r="C6" s="15">
         <f>-Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="15">
         <f>-Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="15">
         <f>-Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="15">
         <f>-Assumptions!$B$10</f>
         <v/>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="15">
         <f>-Assumptions!$B$10</f>
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>Net Cash Flow ($)</t>
-        </is>
-      </c>
-      <c r="B7" s="16">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Net Annual Cash Flow</t>
+        </is>
+      </c>
+      <c r="B7" s="17">
         <f>B4+B5+B6</f>
         <v/>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="17">
         <f>C4+C5+C6</f>
         <v/>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="17">
         <f>D4+D5+D6</f>
         <v/>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="17">
         <f>E4+E5+E6</f>
         <v/>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="17">
         <f>F4+F5+F6</f>
         <v/>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="17">
         <f>G4+G5+G6</f>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Cumulative Cash Flow ($)</t>
-        </is>
-      </c>
-      <c r="B8" s="14">
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Cumulative Nominal Cash Flow</t>
+        </is>
+      </c>
+      <c r="B8" s="15">
         <f>B7</f>
         <v/>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="15">
         <f>B8+C7</f>
         <v/>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="15">
         <f>C8+D7</f>
         <v/>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="15">
         <f>D8+E7</f>
         <v/>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="15">
         <f>E8+F7</f>
         <v/>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="15">
         <f>F8+G7</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Discount Factor</t>
-        </is>
-      </c>
-      <c r="B9" s="17">
-        <f>1/(1+Assumptions!$B$11)^B$3</f>
-        <v/>
-      </c>
-      <c r="C9" s="17">
-        <f>1/(1+Assumptions!$B$11)^C$3</f>
-        <v/>
-      </c>
-      <c r="D9" s="17">
-        <f>1/(1+Assumptions!$B$11)^D$3</f>
-        <v/>
-      </c>
-      <c r="E9" s="17">
-        <f>1/(1+Assumptions!$B$11)^E$3</f>
-        <v/>
-      </c>
-      <c r="F9" s="17">
-        <f>1/(1+Assumptions!$B$11)^F$3</f>
-        <v/>
-      </c>
-      <c r="G9" s="17">
-        <f>1/(1+Assumptions!$B$11)^G$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>PV of Net Cash Flow ($)</t>
-        </is>
-      </c>
-      <c r="B10" s="14">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Present Value Factor</t>
+        </is>
+      </c>
+      <c r="B9" s="18">
+        <f>1/(1+Assumptions!$B$11)^0</f>
+        <v/>
+      </c>
+      <c r="C9" s="18">
+        <f>1/(1+Assumptions!$B$11)^1</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>1/(1+Assumptions!$B$11)^2</f>
+        <v/>
+      </c>
+      <c r="E9" s="18">
+        <f>1/(1+Assumptions!$B$11)^3</f>
+        <v/>
+      </c>
+      <c r="F9" s="18">
+        <f>1/(1+Assumptions!$B$11)^4</f>
+        <v/>
+      </c>
+      <c r="G9" s="18">
+        <f>1/(1+Assumptions!$B$11)^5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Discounted Net Cash Flow (PV)</t>
+        </is>
+      </c>
+      <c r="B10" s="15">
         <f>B7*B9</f>
         <v/>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="15">
         <f>C7*C9</f>
         <v/>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="15">
         <f>D7*D9</f>
         <v/>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="15">
         <f>E7*E9</f>
         <v/>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="15">
         <f>F7*F9</f>
         <v/>
       </c>
-      <c r="G10" s="14">
+      <c r="G10" s="15">
         <f>G7*G9</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Cumulative PV ($)</t>
-        </is>
-      </c>
-      <c r="B11" s="14">
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Cumulative Present Value (NPV Trend)</t>
+        </is>
+      </c>
+      <c r="B11" s="15">
         <f>B10</f>
         <v/>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="15">
         <f>B11+C10</f>
         <v/>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="15">
         <f>C11+D10</f>
         <v/>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="15">
         <f>D11+E10</f>
         <v/>
       </c>
-      <c r="F11" s="14">
+      <c r="F11" s="15">
         <f>E11+F10</f>
         <v/>
       </c>
-      <c r="G11" s="14">
+      <c r="G11" s="15">
         <f>F11+G10</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Key Metrics</t>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>Executive Investment Scorecard Metrics</t>
         </is>
       </c>
       <c r="B14" s="4" t="n"/>
@@ -1277,42 +1330,42 @@
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="5" t="n"/>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Net Present Value (NPV)</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>ROI (Total)</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>Payback Period (Years)</t>
-        </is>
-      </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>Total Net Savings (undiscounted)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="19">
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Internal Return Multiplier (ROI)</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>Calculated Payback Lifecycle</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>Total Net Capital Delta</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="21">
         <f>NPV(Assumptions!$B$11,C7:G7)+B7</f>
         <v/>
       </c>
-      <c r="B16" s="20">
+      <c r="B16" s="22">
         <f>SUM(C7:G7)/-B7</f>
         <v/>
       </c>
-      <c r="C16" s="21">
-        <f>IFERROR(MATCH(TRUE,INDEX(B8:G8&gt;0,0))-2+(-INDEX(B8:G8,MATCH(TRUE,INDEX(B8:G8&gt;0,0))-1))/INDEX(B7:G7,MATCH(TRUE,INDEX(B8:G8&gt;0,0))),"Not within horizon")</f>
-        <v/>
-      </c>
-      <c r="D16" s="19">
+      <c r="C16" s="23">
+        <f>IFERROR(MATCH(TRUE,INDEX(B8:G8&gt;0,0))-2+(-INDEX(B8:G8,MATCH(TRUE,INDEX(B8:G8&gt;0,0))-1))/INDEX(B7:G7,MATCH(TRUE,INDEX(B8:G8&gt;0,0))),"Out of Range")</f>
+        <v/>
+      </c>
+      <c r="D16" s="21">
         <f>SUM(C5:G5)+SUM(C6:G6)</f>
         <v/>
       </c>
@@ -1322,6 +1375,14 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A14:E14"/>
   </mergeCells>
+  <conditionalFormatting sqref="B16">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1333,37 +1394,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>How this model works</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="22" t="inlineStr">
-        <is>
-          <t>1. All inputs live on the 'Assumptions' tab in yellow/blue cells — change any of them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="22" t="inlineStr">
-        <is>
-          <t>2. Year 0 captures one-time implementation and hardware costs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="22" t="inlineStr">
-        <is>
-          <t>3. Remember to click 'Enable Editing' at the top of Excel to load values and chart dimensions.</t>
+          <t>Operational Guidelines &amp; Architectural Design Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>1. Interconnected Architecture: Modifications applied inside the yellow 'Assumptions' tab propagate instantly down calculation layers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>2. Capital Outlay Alignment: Baseline software platforms and ancillary node machinery components aggregate directly into Year 0 outflows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>3. Precision Payback Formula: Calculated fields use true linear index estimation points to establish target breakeven metrics cleanly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>4. Secured Document Notice: Ensure you select 'Enable Editing' in the Microsoft Excel notification ribbons to unlock full local evaluation calculations.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Data: decoupled file profiles to present two unique financial scale scopes
</commit_message>
<xml_diff>
--- a/business_case.xlsx
+++ b/business_case.xlsx
@@ -858,14 +858,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Enterprise Cloud &amp; AI Transformation</t>
+          <t>Warehouse IoT Automation Rollout</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Financial Strategy Proposal | Prepared for: Global Enterprise Corp</t>
+          <t>Financial Strategy Proposal | Prepared for: Acme Logistics Group</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>450000</v>
+        <v>250000</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>125000</v>
+        <v>75000</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>260000</v>
+        <v>130000</v>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>35000</v>
+        <v>15000</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>

</xml_diff>